<commit_message>
fix: capture all XBRL statement tables and reconcile synthetic totals
An audit of the corpus caught two defects in the previous commit.

The rebuilt spreadsheets were far thinner than the SEC-published ones:
a hardcoded R2-R11 range captured ten tables where a 10-K publishes
about seventy. The R-file list is now read from each filing's index.json
rather than guessed, so FY2025 carries 70 sheets against SEC's own 73,
and the 10-Qs carry 44-46. Sheet names are de-duplicated because Excel
truncates at 31 characters and seventy statement titles collide.

The synthetic headcount totals now reconcile against the real figures
each 10-K states on page 8 (161,000 / 164,000 / 166,000), and the
generator raises rather than writing data that contradicts the filings.

Also noted while probing: PDF extraction splits Apple's "full-time
equivalent" across the hyphen as "full- time", so text matching in the
ingest layer must normalise whitespace before comparing.
</commit_message>
<xml_diff>
--- a/data/raw/_synthetic/headcount_by_department.xlsx
+++ b/data/raw/_synthetic/headcount_by_department.xlsx
@@ -540,7 +540,7 @@
         <v>2025</v>
       </c>
       <c r="C9" t="n">
-        <v>63500</v>
+        <v>62500</v>
       </c>
     </row>
     <row r="10">
@@ -553,7 +553,7 @@
         <v>2025</v>
       </c>
       <c r="C10" t="n">
-        <v>29000</v>
+        <v>28500</v>
       </c>
     </row>
     <row r="11">
@@ -566,7 +566,7 @@
         <v>2025</v>
       </c>
       <c r="C11" t="n">
-        <v>33500</v>
+        <v>32500</v>
       </c>
     </row>
     <row r="12">
@@ -579,7 +579,7 @@
         <v>2025</v>
       </c>
       <c r="C12" t="n">
-        <v>22000</v>
+        <v>21500</v>
       </c>
     </row>
     <row r="13">
@@ -592,7 +592,7 @@
         <v>2025</v>
       </c>
       <c r="C13" t="n">
-        <v>11500</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="14">
@@ -605,7 +605,7 @@
         <v>2025</v>
       </c>
       <c r="C14" t="n">
-        <v>10500</v>
+        <v>10000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>